<commit_message>
Updated upto excel utility
</commit_message>
<xml_diff>
--- a/src/test/resources/Readers/Config.xlsx
+++ b/src/test/resources/Readers/Config.xlsx
@@ -1,15 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{56FE3A7D-99D2-4111-B146-1164E48017EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,12 +20,34 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>Row Index</t>
+  </si>
+  <si>
+    <t>testdata</t>
+  </si>
+  <si>
+    <t>Dinoo2#</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -46,13 +70,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +357,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(PGandHostel):Updated with extent report
</commit_message>
<xml_diff>
--- a/src/test/resources/Readers/Config.xlsx
+++ b/src/test/resources/Readers/Config.xlsx
@@ -1,29 +1,79 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30015"/>
+  <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5651D111-3FAF-4C89-AA11-690C053B151F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet3" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>Row Index</t>
+  </si>
+  <si>
+    <t>testdata</t>
+  </si>
+  <si>
+    <t>Dinoo2#</t>
+  </si>
+  <si>
+    <t>LoanAmount</t>
+  </si>
+  <si>
+    <t>Monthly Income</t>
+  </si>
+  <si>
+    <t>Other EMI</t>
+  </si>
+  <si>
+    <t>Rate of Interest</t>
+  </si>
+  <si>
+    <t>Loan Tenure</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -46,13 +96,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +383,83 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC2E0CA1-7DEB-4E36-90A1-5F803F4B8A09}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>478903</v>
+      </c>
+      <c r="B2">
+        <v>60000</v>
+      </c>
+      <c r="C2">
+        <v>54645</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(Packers And Movers)Updated Stepdefinition execution
</commit_message>
<xml_diff>
--- a/src/test/resources/Readers/Config.xlsx
+++ b/src/test/resources/Readers/Config.xlsx
@@ -1,15 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sansa\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C2D379A-B4BF-4A38-BF56-DE0A6F809462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Packers&amp;Movers_Inventory" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,9 +25,68 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+  <si>
+    <t>Row Index</t>
+  </si>
+  <si>
+    <t>testdata</t>
+  </si>
+  <si>
+    <t>Dinoo2#</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>SubCategory</t>
+  </si>
+  <si>
+    <t>Item Name</t>
+  </si>
+  <si>
+    <t>Living Room</t>
+  </si>
+  <si>
+    <t>Chair</t>
+  </si>
+  <si>
+    <t>Arm Chair</t>
+  </si>
+  <si>
+    <t>Bedrooms</t>
+  </si>
+  <si>
+    <t>Kitchen</t>
+  </si>
+  <si>
+    <t>Refrigerator</t>
+  </si>
+  <si>
+    <t>Miscellaneous</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Bicycle Kids</t>
+  </si>
+  <si>
+    <t>Fridge 300-399 lts</t>
+  </si>
+  <si>
+    <t>Air Conditioner</t>
+  </si>
+  <si>
+    <t>Window Air Conditioner (AC)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +94,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,13 +145,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +441,113 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796F08C2-A827-451C-A833-F7EBE30E9E7A}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(Login): resolve element interception issue on login button
</commit_message>
<xml_diff>
--- a/src/test/resources/Readers/Config.xlsx
+++ b/src/test/resources/Readers/Config.xlsx
@@ -1,31 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{BF761388-62DC-4DBA-83A1-29535C42D93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{34371131-0C73-43D9-A652-A6E385DE4EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:L32"/>
+  <oleSize ref="A1:K24"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t>Row Index</t>
   </si>
@@ -64,13 +63,73 @@
   </si>
   <si>
     <t>wert@gmail.com</t>
+  </si>
+  <si>
+    <t>LoanAmount</t>
+  </si>
+  <si>
+    <t>Monthly Income</t>
+  </si>
+  <si>
+    <t>Other EMI</t>
+  </si>
+  <si>
+    <t>Rate of Interest</t>
+  </si>
+  <si>
+    <t>Loan Tenure</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>SubCategory</t>
+  </si>
+  <si>
+    <t>Item Name</t>
+  </si>
+  <si>
+    <t>Living Room</t>
+  </si>
+  <si>
+    <t>Chair</t>
+  </si>
+  <si>
+    <t>Arm Chair</t>
+  </si>
+  <si>
+    <t>Bedrooms</t>
+  </si>
+  <si>
+    <t>Air Conditioner</t>
+  </si>
+  <si>
+    <t>Window Air Conditioner (AC)</t>
+  </si>
+  <si>
+    <t>Kitchen</t>
+  </si>
+  <si>
+    <t>Refrigerator</t>
+  </si>
+  <si>
+    <t>Fridge 300-399 lts</t>
+  </si>
+  <si>
+    <t>Miscellaneous</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Bicycle Kids</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,13 +145,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -108,10 +192,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -394,13 +487,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -408,7 +501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -425,17 +518,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F987D82D-7128-4822-82C1-346CA3D3D130}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" customWidth="1"/>
+    <col min="6" max="6" width="21.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -455,7 +548,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -482,4 +575,129 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7942549A-3E07-4304-BCCD-225AF16D66CE}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>478903</v>
+      </c>
+      <c r="B2">
+        <v>60000</v>
+      </c>
+      <c r="C2">
+        <v>54645</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190909F-22C2-43F5-B0CC-A6C73E12030F}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>